<commit_message>
Cover mixed column sorting and guarded Excel oracle cleanup
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/sort-collation.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/sort-collation.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\przemyslaw.klys.EVOTEC\.codex\worktrees\excel-csv-quality\OfficeIMO\OfficeIMO.TestAssets\Documents\ExcelFormulaCorpus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DC6DD97-0807-4C25-AFAD-5CD8542B5131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE001441-B23D-42ED-9FB0-3B508AB76B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="16170" windowWidth="28996" windowHeight="15675" xr2:uid="{F1F8C4F9-CDD6-4F47-BD34-CFEF8163802C}"/>
+    <workbookView xWindow="-98" yWindow="16170" windowWidth="28996" windowHeight="15675" xr2:uid="{D67C1B86-BAA6-48C7-AC3B-BF25F2D37C9E}"/>
   </bookViews>
   <sheets>
-    <sheet name="TextCaseTies" sheetId="12" r:id="rId1"/>
-    <sheet name="TextByColumns" sheetId="11" r:id="rId2"/>
-    <sheet name="BlankTextDescending" sheetId="10" r:id="rId3"/>
-    <sheet name="BlankText" sheetId="9" r:id="rId4"/>
-    <sheet name="MixedBooleanDescending" sheetId="8" r:id="rId5"/>
-    <sheet name="MixedBoolean" sheetId="7" r:id="rId6"/>
-    <sheet name="MixedDescending" sheetId="6" r:id="rId7"/>
-    <sheet name="MixedKeys" sheetId="5" r:id="rId8"/>
-    <sheet name="BlankNumericDescending" sheetId="4" r:id="rId9"/>
-    <sheet name="BlankNumeric" sheetId="3" r:id="rId10"/>
-    <sheet name="TextDescending" sheetId="2" r:id="rId11"/>
-    <sheet name="TextAscending" sheetId="1" r:id="rId12"/>
+    <sheet name="TextCaseTies" sheetId="13" r:id="rId1"/>
+    <sheet name="MixedByColumnsDescending" sheetId="12" r:id="rId2"/>
+    <sheet name="TextByColumns" sheetId="11" r:id="rId3"/>
+    <sheet name="BlankTextDescending" sheetId="10" r:id="rId4"/>
+    <sheet name="BlankText" sheetId="9" r:id="rId5"/>
+    <sheet name="MixedBooleanDescending" sheetId="8" r:id="rId6"/>
+    <sheet name="MixedBoolean" sheetId="7" r:id="rId7"/>
+    <sheet name="MixedDescending" sheetId="6" r:id="rId8"/>
+    <sheet name="MixedKeys" sheetId="5" r:id="rId9"/>
+    <sheet name="BlankNumericDescending" sheetId="4" r:id="rId10"/>
+    <sheet name="BlankNumeric" sheetId="3" r:id="rId11"/>
+    <sheet name="TextDescending" sheetId="2" r:id="rId12"/>
+    <sheet name="TextAscending" sheetId="1" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -72,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="7">
   <si>
     <t>pear</t>
   </si>
@@ -464,7 +465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36E18962-0B2E-4A28-AA7C-CD65BA4119BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BCD05CE-57E8-436F-80BD-0519CB935387}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -520,7 +521,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0511C1BD-AE35-4267-B36C-0A491362E6B1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D0D947-CF74-48F8-A742-C9407B79A4AA}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -534,11 +535,11 @@
         <v>1</v>
       </c>
       <c r="G1" cm="1">
-        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,1)</f>
-        <v>1</v>
+        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,-1)</f>
+        <v>2</v>
       </c>
       <c r="H1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -547,10 +548,10 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -575,7 +576,62 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA86394-6364-4B48-AA4B-01E89F725B36}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE577D01-34F8-468A-AA2E-D0972D037CB3}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" cm="1">
+        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,1)</f>
+        <v>1</v>
+      </c>
+      <c r="H1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89E2940-DDFA-47C1-A64E-E67ED684E305}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -630,8 +686,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84B1CD70-5213-4939-85F3-E4F5DDD8223B}">
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E20F1E40-545C-4F01-8BDA-6F9E8DF90119}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -687,7 +743,87 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D47C110E-BD0A-443E-9606-E4EA3041D337}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C08C2F-A7E1-4414-B629-2CA401DBF452}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="b">
+        <f>FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="D1" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="G1" t="b" cm="1">
+        <f t="array" ref="G1:K2">_xlfn._xlws.SORT(A1:E2,1,-1,TRUE)</f>
+        <v>1</v>
+      </c>
+      <c r="H1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1" t="str">
+        <v>a</v>
+      </c>
+      <c r="J1">
+        <v>1</v>
+      </c>
+      <c r="K1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BB3206B-8F59-4F2C-BE51-6E9EB5C3BAD4}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -740,8 +876,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A635E22D-A6C4-41F5-8196-FB9C577ABC40}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BAD580C-E63C-4634-9CFB-0A8B5299E768}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -793,8 +929,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF365ED8-F1AE-491E-9F61-5484D3211171}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A528EA95-DEFE-4F32-B15A-93FD6B697B67}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -846,8 +982,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38176E14-0991-4529-A4CC-99BF66AEDC67}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B48DDD-297F-4572-BA35-071425547ECC}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -932,8 +1068,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAFE7114-4F3A-4F1C-9279-C077024150EE}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E69F423-867A-4B17-BD16-484FAF21F524}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1018,8 +1154,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19330BC7-75E1-4666-9BD3-B4EE102C1752}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16D435F2-0576-4260-A6E4-AE323AD08296}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1091,8 +1227,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FAC118A-BC55-4546-8F0D-F9F531F995CE}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2210C602-413B-49C2-BAB6-540D37C19B03}">
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1162,59 +1298,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9B71973-86CC-4054-A307-77AEEDB54242}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="B1">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G1" cm="1">
-        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,-1)</f>
-        <v>2</v>
-      </c>
-      <c r="H1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B2">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Qualify ASCII digit text SORT keys against Excel
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/sort-collation.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/sort-collation.xlsx
@@ -8,24 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\przemyslaw.klys.EVOTEC\.codex\worktrees\excel-csv-quality\OfficeIMO\OfficeIMO.TestAssets\Documents\ExcelFormulaCorpus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE001441-B23D-42ED-9FB0-3B508AB76B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B1BF2A8-6087-4412-8BD4-6C0E699C9A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="16170" windowWidth="28996" windowHeight="15675" xr2:uid="{D67C1B86-BAA6-48C7-AC3B-BF25F2D37C9E}"/>
+    <workbookView xWindow="-98" yWindow="16170" windowWidth="28996" windowHeight="15675" xr2:uid="{63EB1896-1540-4244-9290-03E8BC8BE048}"/>
   </bookViews>
   <sheets>
-    <sheet name="TextCaseTies" sheetId="13" r:id="rId1"/>
-    <sheet name="MixedByColumnsDescending" sheetId="12" r:id="rId2"/>
-    <sheet name="TextByColumns" sheetId="11" r:id="rId3"/>
-    <sheet name="BlankTextDescending" sheetId="10" r:id="rId4"/>
-    <sheet name="BlankText" sheetId="9" r:id="rId5"/>
-    <sheet name="MixedBooleanDescending" sheetId="8" r:id="rId6"/>
-    <sheet name="MixedBoolean" sheetId="7" r:id="rId7"/>
-    <sheet name="MixedDescending" sheetId="6" r:id="rId8"/>
-    <sheet name="MixedKeys" sheetId="5" r:id="rId9"/>
-    <sheet name="BlankNumericDescending" sheetId="4" r:id="rId10"/>
-    <sheet name="BlankNumeric" sheetId="3" r:id="rId11"/>
-    <sheet name="TextDescending" sheetId="2" r:id="rId12"/>
-    <sheet name="TextAscending" sheetId="1" r:id="rId13"/>
+    <sheet name="PunctuationText" sheetId="16" r:id="rId1"/>
+    <sheet name="NumericText" sheetId="15" r:id="rId2"/>
+    <sheet name="DigitText" sheetId="14" r:id="rId3"/>
+    <sheet name="TextCaseTies" sheetId="13" r:id="rId4"/>
+    <sheet name="MixedByColumnsDescending" sheetId="12" r:id="rId5"/>
+    <sheet name="TextByColumns" sheetId="11" r:id="rId6"/>
+    <sheet name="BlankTextDescending" sheetId="10" r:id="rId7"/>
+    <sheet name="BlankText" sheetId="9" r:id="rId8"/>
+    <sheet name="MixedBooleanDescending" sheetId="8" r:id="rId9"/>
+    <sheet name="MixedBoolean" sheetId="7" r:id="rId10"/>
+    <sheet name="MixedDescending" sheetId="6" r:id="rId11"/>
+    <sheet name="MixedKeys" sheetId="5" r:id="rId12"/>
+    <sheet name="BlankNumericDescending" sheetId="4" r:id="rId13"/>
+    <sheet name="BlankNumeric" sheetId="3" r:id="rId14"/>
+    <sheet name="TextDescending" sheetId="2" r:id="rId15"/>
+    <sheet name="TextAscending" sheetId="1" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -73,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
   <si>
     <t>pear</t>
   </si>
@@ -94,6 +97,51 @@
   </si>
   <si>
     <t>APPLE</t>
+  </si>
+  <si>
+    <t>v2</t>
+  </si>
+  <si>
+    <t>v10</t>
+  </si>
+  <si>
+    <t>v1</t>
+  </si>
+  <si>
+    <t>v02</t>
+  </si>
+  <si>
+    <t>v9</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>a-b</t>
+  </si>
+  <si>
+    <t>a_b</t>
+  </si>
+  <si>
+    <t>ab</t>
+  </si>
+  <si>
+    <t>a b</t>
+  </si>
+  <si>
+    <t>a.b</t>
   </si>
 </sst>
 </file>
@@ -130,8 +178,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,21 +514,449 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BCD05CE-57E8-436F-80BD-0519CB935387}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8821F410-26B7-4F36-88A0-791E7C4F3A59}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" t="str" cm="1">
+        <f t="array" ref="G1:H5">_xlfn._xlws.SORT(A1:B5,1,1)</f>
+        <v>a b</v>
+      </c>
+      <c r="H1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>a.b</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>a_b</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>ab</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="G5" t="str">
+        <v>a-b</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C06255B-AED8-41ED-8232-B5646D46D9A2}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="b">
+        <f>FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" cm="1">
+        <f t="array" ref="G1:H5">_xlfn._xlws.SORT(A1:B5,1,1)</f>
+        <v>1</v>
+      </c>
+      <c r="H1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>a</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B5">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA41469-0A3B-4200-AC29-88E43F3717B0}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" t="str" cm="1">
+        <f t="array" ref="G1:H4">_xlfn._xlws.SORT(A1:B4,1,-1)</f>
+        <v>b</v>
+      </c>
+      <c r="H1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>a</v>
+      </c>
+      <c r="H2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0B85FA7-D3A8-4056-B334-361E11DF921A}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" cm="1">
+        <f t="array" ref="G1:H4">_xlfn._xlws.SORT(A1:B4,1,1)</f>
+        <v>1</v>
+      </c>
+      <c r="H1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>a</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>b</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4255050-B8BB-4A2B-B5B1-1E01CC7DCC40}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" cm="1">
+        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,-1)</f>
+        <v>2</v>
+      </c>
+      <c r="H1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B036777-0A20-4978-8F5B-380E56AE99FC}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" cm="1">
+        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,1)</f>
+        <v>1</v>
+      </c>
+      <c r="H1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{405C41E3-4E77-40E4-87DF-254FEB74F6BA}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1">
         <f>1</f>
         <v>1</v>
       </c>
       <c r="G1" t="str" cm="1">
-        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,1)</f>
-        <v>apple</v>
+        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,-1)</f>
+        <v>pear</v>
       </c>
       <c r="H1">
         <v>1</v>
@@ -487,32 +964,32 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <f>2</f>
         <v>2</v>
       </c>
       <c r="G2" t="str">
-        <v>Apple</v>
+        <v>banana</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <f>3</f>
         <v>3</v>
       </c>
       <c r="G3" t="str">
-        <v>APPLE</v>
+        <v>apple</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -520,118 +997,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8D0D947-CF74-48F8-A742-C9407B79A4AA}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="B1">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G1" cm="1">
-        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,-1)</f>
-        <v>2</v>
-      </c>
-      <c r="H1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B2">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE577D01-34F8-468A-AA2E-D0972D037CB3}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="B1">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G1" cm="1">
-        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,1)</f>
-        <v>1</v>
-      </c>
-      <c r="H1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B2">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E89E2940-DDFA-47C1-A64E-E67ED684E305}">
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F4AC01E-022D-47F6-B7A7-EA30FBBE05AC}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -644,11 +1011,11 @@
         <v>1</v>
       </c>
       <c r="G1" t="str" cm="1">
-        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,-1)</f>
-        <v>pear</v>
+        <f t="array" ref="G1:H3">_xlfn._xlws.SORT(A1:B3,1,1)</f>
+        <v>apple</v>
       </c>
       <c r="H1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -675,10 +1042,10 @@
         <v>3</v>
       </c>
       <c r="G3" t="str">
-        <v>apple</v>
+        <v>pear</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -686,14 +1053,186 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E20F1E40-545C-4F01-8BDA-6F9E8DF90119}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12664808-3D00-4F97-8FBA-DB0936EE4F42}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" t="str" cm="1">
+        <f t="array" ref="G1:H5">_xlfn._xlws.SORT(A1:B5,1,1)</f>
+        <v>02</v>
+      </c>
+      <c r="H1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>10</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="G5" t="str">
+        <v>9</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB083F2E-5BAF-462B-A758-F641B455A50D}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="G1" t="str" cm="1">
+        <f t="array" ref="G1:H5">_xlfn._xlws.SORT(A1:B5,1,1)</f>
+        <v>v02</v>
+      </c>
+      <c r="H1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>v1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <f>3</f>
+        <v>3</v>
+      </c>
+      <c r="G3" t="str">
+        <v>v10</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <f>4</f>
+        <v>4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>v2</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <f>5</f>
+        <v>5</v>
+      </c>
+      <c r="G5" t="str">
+        <v>v9</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E92DBED8-000A-49E6-AA44-E3DB78B334F6}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1">
         <f>1</f>
@@ -704,37 +1243,37 @@
         <v>apple</v>
       </c>
       <c r="H1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <f>2</f>
         <v>2</v>
       </c>
       <c r="G2" t="str">
-        <v>banana</v>
+        <v>Apple</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <f>3</f>
         <v>3</v>
       </c>
       <c r="G3" t="str">
-        <v>pear</v>
+        <v>APPLE</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -742,8 +1281,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C08C2F-A7E1-4414-B629-2CA401DBF452}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7CF99B4-539C-4330-B8C6-43C70ED15D23}">
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -822,8 +1361,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BB3206B-8F59-4F2C-BE51-6E9EB5C3BAD4}">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB12BE7F-9628-4875-9E96-DEDE6CEC1E8B}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -876,8 +1415,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BAD580C-E63C-4634-9CFB-0A8B5299E768}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66064C8C-877A-4DB2-B5D5-2FA775A5BFE1}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -929,8 +1468,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A528EA95-DEFE-4F32-B15A-93FD6B697B67}">
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB9300AC-BCBC-4397-9A7B-FA1BB4D526A9}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -982,8 +1521,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75B48DDD-297F-4572-BA35-071425547ECC}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D39A5904-2D75-48C5-9C6E-D73C7B3D43BC}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
@@ -1066,236 +1605,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E69F423-867A-4B17-BD16-484FAF21F524}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="b">
-        <f>FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G1" cm="1">
-        <f t="array" ref="G1:H5">_xlfn._xlws.SORT(A1:B5,1,1)</f>
-        <v>1</v>
-      </c>
-      <c r="H1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="G2" t="str">
-        <v>a</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="G3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="b">
-        <f>TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <f>4</f>
-        <v>4</v>
-      </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B5">
-        <f>5</f>
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16D435F2-0576-4260-A6E4-AE323AD08296}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="B1">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G1" t="str" cm="1">
-        <f t="array" ref="G1:H4">_xlfn._xlws.SORT(A1:B4,1,-1)</f>
-        <v>b</v>
-      </c>
-      <c r="H1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="G2" t="str">
-        <v>a</v>
-      </c>
-      <c r="H2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <f>4</f>
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2210C602-413B-49C2-BAB6-540D37C19B03}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="B1">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G1" cm="1">
-        <f t="array" ref="G1:H4">_xlfn._xlws.SORT(A1:B4,1,1)</f>
-        <v>1</v>
-      </c>
-      <c r="H1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <f>3</f>
-        <v>3</v>
-      </c>
-      <c r="G3" t="str">
-        <v>a</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <f>4</f>
-        <v>4</v>
-      </c>
-      <c r="G4" t="str">
-        <v>b</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>